<commit_message>
made the pages instance from static
</commit_message>
<xml_diff>
--- a/Data/RegressionUI.xlsx
+++ b/Data/RegressionUI.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/harshverma/IdeaProjects/AutomationPack/Data/"/>
     </mc:Choice>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="22">
   <si>
     <t>Run</t>
   </si>
@@ -109,6 +109,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -466,82 +467,82 @@
   <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="38.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.33203125" customWidth="1"/>
-    <col min="6" max="6" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="38.5"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="14.33203125"/>
+    <col min="5" max="5" customWidth="true" width="14.33203125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="13.57421875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>5</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>10</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="0">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2">
+      <c r="A2" s="0">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>3</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="0">
         <v>9</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="0">
         <v>8</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" t="s" s="0">
         <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3">
+      <c r="A3" s="0">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="B3" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s" s="0">
         <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4">
+      <c r="A4" s="0">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="B4" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C4" t="s" s="0">
         <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="A5" s="0">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s" s="0">
         <v>8</v>
       </c>
     </row>
@@ -556,18 +557,18 @@
   <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="12.6640625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="13.5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>10</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -576,15 +577,15 @@
       <c r="E1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="0">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2">
+      <c r="A2" s="0">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>3</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -596,31 +597,31 @@
       <c r="E2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" t="s" s="0">
         <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3">
+      <c r="A3" s="0">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4">
+      <c r="A4" s="0">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" t="s" s="0">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="A5" s="0">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s" s="0">
         <v>4</v>
       </c>
     </row>
@@ -635,38 +636,38 @@
   <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="5" max="5" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="11.1640625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="13.5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>16</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="0">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2">
+      <c r="A2" s="0">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>3</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" t="s" s="0">
         <v>21</v>
       </c>
       <c r="D2" s="1" t="s">
@@ -675,31 +676,31 @@
       <c r="E2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" t="s" s="0">
         <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3">
+      <c r="A3" s="0">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4">
+      <c r="A4" s="0">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" t="s" s="0">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="A5" s="0">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s" s="0">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added file upload method
</commit_message>
<xml_diff>
--- a/Data/RegressionUI.xlsx
+++ b/Data/RegressionUI.xlsx
@@ -3,23 +3,24 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/harshverma/IdeaProjects/AutomationPack/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7BF5658-3A3B-6944-ABC7-C77E21779AB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9273689B-3F7B-5442-AE76-E8F5DF2D272C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1360" yWindow="740" windowWidth="28040" windowHeight="16620" activeTab="1" xr2:uid="{6B8C0FC8-8986-4A42-A027-2171E9EAAECE}"/>
+    <workbookView xWindow="1360" yWindow="740" windowWidth="28040" windowHeight="16620" activeTab="2" xr2:uid="{6B8C0FC8-8986-4A42-A027-2171E9EAAECE}"/>
   </bookViews>
   <sheets>
     <sheet name="timeSheet" sheetId="1" r:id="rId1"/>
     <sheet name="attendance" sheetId="2" r:id="rId2"/>
-    <sheet name="pimUpdate" sheetId="3" r:id="rId3"/>
+    <sheet name="admin" sheetId="4" r:id="rId3"/>
+    <sheet name="pimUpdate" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="23">
   <si>
     <t>Run</t>
   </si>
@@ -103,13 +104,15 @@
   </si>
   <si>
     <t>ninja</t>
+  </si>
+  <si>
+    <t>clientLogo</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -467,82 +470,82 @@
   <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="38.5"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="14.33203125"/>
-    <col min="5" max="5" customWidth="true" width="14.33203125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="13.57421875"/>
+    <col min="3" max="3" width="38.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.33203125" customWidth="1"/>
+    <col min="6" max="6" width="13.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>5</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>10</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="0">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s" s="0">
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s" s="0">
+      <c r="D2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="0">
+      <c r="E2">
         <v>8</v>
       </c>
-      <c r="F2" t="s" s="0">
+      <c r="F2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="0">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="C3" t="s" s="0">
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="0">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="C4" t="s" s="0">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="0">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="C5" t="s" s="0">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
         <v>8</v>
       </c>
     </row>
@@ -557,18 +560,18 @@
   <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="12.6640625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="13.5"/>
+    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>10</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -577,15 +580,15 @@
       <c r="E1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="0">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -597,31 +600,31 @@
       <c r="E2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F2" t="s" s="0">
+      <c r="F2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="0">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="0">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s" s="0">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="0">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s" s="0">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
         <v>4</v>
       </c>
     </row>
@@ -632,42 +635,104 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6E4E407-5143-A04B-AD03-75A73E998080}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{275B3916-9281-9B4E-9587-223060CB0ABA}">
   <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="11.1640625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="13.5"/>
+    <col min="5" max="5" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>16</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="0">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s" s="0">
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
         <v>21</v>
       </c>
       <c r="D2" s="1" t="s">
@@ -676,31 +741,31 @@
       <c r="E2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F2" t="s" s="0">
+      <c r="F2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="0">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="0">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s" s="0">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="0">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s" s="0">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>